<commit_message>
Estimacion de Gastos / comisiones y variables
</commit_message>
<xml_diff>
--- a/storage/app/public/glosario.xlsx
+++ b/storage/app/public/glosario.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="779" uniqueCount="512">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="809" uniqueCount="523">
   <si>
     <t xml:space="preserve">utiliza_transporte</t>
   </si>
@@ -809,7 +809,7 @@
     <t xml:space="preserve">Analista De Planificación Y Control De Gestion</t>
   </si>
   <si>
-    <t xml:space="preserve">Redes Sociales (RRSS)</t>
+    <t xml:space="preserve">Redes Sociales (rrss)</t>
   </si>
   <si>
     <t xml:space="preserve">la rinconada</t>
@@ -1409,52 +1409,85 @@
     <t xml:space="preserve">Asistente de Marca</t>
   </si>
   <si>
+    <t xml:space="preserve">Kia</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Kia Encuestas</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ejecutivo Comercial</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Librepago G</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Backoffice de Mercadeo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Di Stasi Motors G</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Asesor Comercial</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Corpocredit G</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Supervisor de Ventas</t>
+  </si>
+  <si>
+    <t xml:space="preserve">G-talent</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Coordinadora de Captación y Selección de  Talentos</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ubii Pagos Cobranzas</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Coordinador de Mercadeo y RRPP</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Oceanica De Seguros</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ventas Oceanica De Seguros</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Analista de Back Office</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cobranzas Oceanica De Seguros</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Supervisor Senior de BackOffice</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Jac Motors</t>
+  </si>
+  <si>
     <t xml:space="preserve">Gerencia de Formacion y Calidad</t>
   </si>
   <si>
     <t xml:space="preserve">Formación</t>
   </si>
   <si>
-    <t xml:space="preserve">Ejecutivo Comercial</t>
-  </si>
-  <si>
     <t xml:space="preserve">Calidad</t>
   </si>
   <si>
-    <t xml:space="preserve">Backoffice de Mercadeo</t>
-  </si>
-  <si>
     <t xml:space="preserve">Captación</t>
   </si>
   <si>
-    <t xml:space="preserve">Asesor Comercial</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Supervisor de Ventas</t>
-  </si>
-  <si>
     <t xml:space="preserve">Gerencia Business Intelligence</t>
   </si>
   <si>
-    <t xml:space="preserve">Coordinadora de Captación y Selección de  Talentos</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Coordinador de Mercadeo y RRPP</t>
-  </si>
-  <si>
     <t xml:space="preserve">Backoffice</t>
   </si>
   <si>
     <t xml:space="preserve">Backoficce</t>
   </si>
   <si>
-    <t xml:space="preserve">Analista de Back Office</t>
-  </si>
-  <si>
     <t xml:space="preserve">Formacion</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Supervisor Senior de BackOffice</t>
   </si>
   <si>
     <t xml:space="preserve">Gerencia De Tecnología</t>
@@ -1979,7 +2012,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:AM145"/>
+  <dimension ref="A1:AM154"/>
   <sheetFormatPr defaultColWidth="11.640625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="17.67"/>
@@ -5041,10 +5074,10 @@
         <v>461</v>
       </c>
       <c r="AI125" s="15" t="s">
+        <v>51</v>
+      </c>
+      <c r="AJ125" s="15" t="s">
         <v>462</v>
-      </c>
-      <c r="AJ125" s="15" t="s">
-        <v>36</v>
       </c>
       <c r="AK125" s="15" t="s">
         <v>463</v>
@@ -5055,10 +5088,10 @@
         <v>464</v>
       </c>
       <c r="AI126" s="15" t="s">
-        <v>462</v>
+        <v>51</v>
       </c>
       <c r="AJ126" s="15" t="s">
-        <v>36</v>
+        <v>465</v>
       </c>
       <c r="AK126" s="15" t="s">
         <v>465</v>
@@ -5069,10 +5102,10 @@
         <v>466</v>
       </c>
       <c r="AI127" s="15" t="s">
-        <v>462</v>
+        <v>51</v>
       </c>
       <c r="AJ127" s="15" t="s">
-        <v>36</v>
+        <v>467</v>
       </c>
       <c r="AK127" s="15" t="s">
         <v>467</v>
@@ -5083,116 +5116,116 @@
         <v>468</v>
       </c>
       <c r="AI128" s="15" t="s">
-        <v>462</v>
+        <v>51</v>
       </c>
       <c r="AJ128" s="15" t="s">
-        <v>36</v>
+        <v>469</v>
       </c>
       <c r="AK128" s="15" t="s">
-        <v>352</v>
+        <v>469</v>
       </c>
     </row>
     <row r="129" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G129" s="1" t="s">
-        <v>469</v>
+        <v>470</v>
       </c>
       <c r="AI129" s="15" t="s">
-        <v>470</v>
+        <v>51</v>
       </c>
       <c r="AJ129" s="15" t="s">
-        <v>36</v>
+        <v>471</v>
       </c>
       <c r="AK129" s="15" t="s">
-        <v>36</v>
+        <v>471</v>
       </c>
     </row>
     <row r="130" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G130" s="1" t="s">
-        <v>471</v>
+        <v>472</v>
       </c>
       <c r="AI130" s="15" t="s">
-        <v>470</v>
+        <v>51</v>
       </c>
       <c r="AJ130" s="15" t="s">
-        <v>36</v>
+        <v>473</v>
       </c>
       <c r="AK130" s="15" t="s">
-        <v>352</v>
+        <v>473</v>
       </c>
     </row>
     <row r="131" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G131" s="1" t="s">
-        <v>472</v>
+        <v>474</v>
       </c>
       <c r="AI131" s="15" t="s">
-        <v>470</v>
+        <v>51</v>
       </c>
       <c r="AJ131" s="15" t="s">
-        <v>473</v>
+        <v>475</v>
       </c>
       <c r="AK131" s="15" t="s">
-        <v>474</v>
+        <v>476</v>
       </c>
     </row>
     <row r="132" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G132" s="1" t="s">
+        <v>477</v>
+      </c>
+      <c r="AI132" s="15" t="s">
+        <v>51</v>
+      </c>
+      <c r="AJ132" s="15" t="s">
         <v>475</v>
       </c>
-      <c r="AI132" s="15" t="s">
-        <v>470</v>
-      </c>
-      <c r="AJ132" s="15" t="s">
-        <v>476</v>
-      </c>
       <c r="AK132" s="15" t="s">
-        <v>476</v>
+        <v>478</v>
       </c>
     </row>
     <row r="133" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G133" s="1" t="s">
-        <v>477</v>
+        <v>479</v>
       </c>
       <c r="AI133" s="15" t="s">
-        <v>478</v>
+        <v>51</v>
       </c>
       <c r="AJ133" s="15" t="s">
-        <v>36</v>
+        <v>480</v>
       </c>
       <c r="AK133" s="15" t="s">
-        <v>36</v>
+        <v>480</v>
       </c>
     </row>
     <row r="134" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="AI134" s="15" t="s">
-        <v>478</v>
+        <v>51</v>
       </c>
       <c r="AJ134" s="15" t="s">
-        <v>36</v>
+        <v>480</v>
       </c>
       <c r="AK134" s="15" t="s">
-        <v>352</v>
+        <v>480</v>
       </c>
     </row>
     <row r="135" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="AI135" s="15" t="s">
-        <v>479</v>
+        <v>481</v>
       </c>
       <c r="AJ135" s="15" t="s">
         <v>36</v>
       </c>
       <c r="AK135" s="15" t="s">
-        <v>36</v>
+        <v>482</v>
       </c>
     </row>
     <row r="136" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="AI136" s="15" t="s">
-        <v>480</v>
+        <v>481</v>
       </c>
       <c r="AJ136" s="15" t="s">
         <v>36</v>
       </c>
       <c r="AK136" s="15" t="s">
-        <v>36</v>
+        <v>483</v>
       </c>
     </row>
     <row r="137" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5203,23 +5236,23 @@
         <v>36</v>
       </c>
       <c r="AK137" s="15" t="s">
-        <v>36</v>
+        <v>484</v>
       </c>
     </row>
     <row r="138" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="AI138" s="15" t="s">
-        <v>482</v>
+        <v>481</v>
       </c>
       <c r="AJ138" s="15" t="s">
         <v>36</v>
       </c>
       <c r="AK138" s="15" t="s">
-        <v>36</v>
+        <v>352</v>
       </c>
     </row>
     <row r="139" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="AI139" s="15" t="s">
-        <v>483</v>
+        <v>485</v>
       </c>
       <c r="AJ139" s="15" t="s">
         <v>36</v>
@@ -5230,13 +5263,13 @@
     </row>
     <row r="140" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="AI140" s="15" t="s">
-        <v>484</v>
+        <v>485</v>
       </c>
       <c r="AJ140" s="15" t="s">
         <v>36</v>
       </c>
       <c r="AK140" s="15" t="s">
-        <v>36</v>
+        <v>352</v>
       </c>
     </row>
     <row r="141" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5244,26 +5277,26 @@
         <v>485</v>
       </c>
       <c r="AJ141" s="15" t="s">
-        <v>36</v>
+        <v>486</v>
       </c>
       <c r="AK141" s="15" t="s">
-        <v>36</v>
+        <v>487</v>
       </c>
     </row>
     <row r="142" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="AI142" s="15" t="s">
-        <v>486</v>
+        <v>485</v>
       </c>
       <c r="AJ142" s="15" t="s">
-        <v>36</v>
+        <v>488</v>
       </c>
       <c r="AK142" s="15" t="s">
-        <v>36</v>
+        <v>488</v>
       </c>
     </row>
     <row r="143" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="AI143" s="15" t="s">
-        <v>487</v>
+        <v>489</v>
       </c>
       <c r="AJ143" s="15" t="s">
         <v>36</v>
@@ -5274,19 +5307,124 @@
     </row>
     <row r="144" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="AI144" s="15" t="s">
-        <v>488</v>
+        <v>489</v>
       </c>
       <c r="AJ144" s="15" t="s">
-        <v>489</v>
+        <v>36</v>
       </c>
       <c r="AK144" s="15" t="s">
+        <v>352</v>
+      </c>
+    </row>
+    <row r="145" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="AI145" s="15" t="s">
+        <v>490</v>
+      </c>
+      <c r="AJ145" s="15" t="s">
         <v>36</v>
       </c>
-    </row>
-    <row r="145" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="AI145" s="15"/>
-      <c r="AJ145" s="15"/>
-      <c r="AK145" s="15"/>
+      <c r="AK145" s="15" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="146" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="AI146" s="15" t="s">
+        <v>491</v>
+      </c>
+      <c r="AJ146" s="15" t="s">
+        <v>36</v>
+      </c>
+      <c r="AK146" s="15" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="147" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="AI147" s="15" t="s">
+        <v>492</v>
+      </c>
+      <c r="AJ147" s="15" t="s">
+        <v>36</v>
+      </c>
+      <c r="AK147" s="15" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="148" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="AI148" s="15" t="s">
+        <v>493</v>
+      </c>
+      <c r="AJ148" s="15" t="s">
+        <v>36</v>
+      </c>
+      <c r="AK148" s="15" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="149" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="AI149" s="15" t="s">
+        <v>494</v>
+      </c>
+      <c r="AJ149" s="15" t="s">
+        <v>36</v>
+      </c>
+      <c r="AK149" s="15" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="150" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="AI150" s="15" t="s">
+        <v>495</v>
+      </c>
+      <c r="AJ150" s="15" t="s">
+        <v>36</v>
+      </c>
+      <c r="AK150" s="15" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="151" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="AI151" s="15" t="s">
+        <v>496</v>
+      </c>
+      <c r="AJ151" s="15" t="s">
+        <v>36</v>
+      </c>
+      <c r="AK151" s="15" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="152" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="AI152" s="15" t="s">
+        <v>497</v>
+      </c>
+      <c r="AJ152" s="15" t="s">
+        <v>36</v>
+      </c>
+      <c r="AK152" s="15" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="153" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="AI153" s="15" t="s">
+        <v>498</v>
+      </c>
+      <c r="AJ153" s="15" t="s">
+        <v>36</v>
+      </c>
+      <c r="AK153" s="15" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="154" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="AI154" s="15" t="s">
+        <v>499</v>
+      </c>
+      <c r="AJ154" s="15" t="s">
+        <v>500</v>
+      </c>
+      <c r="AK154" s="15" t="s">
+        <v>36</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -5315,7 +5453,7 @@
         <v>1</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>490</v>
+        <v>501</v>
       </c>
       <c r="D1" s="1" t="n">
         <v>1</v>
@@ -5326,7 +5464,7 @@
         <v>2</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>491</v>
+        <v>502</v>
       </c>
       <c r="D2" s="1" t="n">
         <v>1</v>
@@ -5337,7 +5475,7 @@
         <v>3</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>492</v>
+        <v>503</v>
       </c>
       <c r="D3" s="1" t="n">
         <v>1</v>
@@ -5348,7 +5486,7 @@
         <v>4</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>493</v>
+        <v>504</v>
       </c>
       <c r="D4" s="1" t="n">
         <v>1</v>
@@ -5359,7 +5497,7 @@
         <v>5</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>494</v>
+        <v>505</v>
       </c>
       <c r="D5" s="1" t="n">
         <v>1</v>
@@ -5370,7 +5508,7 @@
         <v>6</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>495</v>
+        <v>506</v>
       </c>
       <c r="D6" s="1" t="n">
         <v>1</v>
@@ -5381,7 +5519,7 @@
         <v>7</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>496</v>
+        <v>507</v>
       </c>
       <c r="D7" s="1" t="n">
         <v>1</v>
@@ -5392,7 +5530,7 @@
         <v>8</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>490</v>
+        <v>501</v>
       </c>
       <c r="D8" s="1" t="n">
         <v>1</v>
@@ -5403,7 +5541,7 @@
         <v>9</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>497</v>
+        <v>508</v>
       </c>
       <c r="D9" s="1" t="n">
         <v>1</v>
@@ -5414,7 +5552,7 @@
         <v>10</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>498</v>
+        <v>509</v>
       </c>
       <c r="D10" s="1" t="n">
         <v>1</v>
@@ -5425,7 +5563,7 @@
         <v>11</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>499</v>
+        <v>510</v>
       </c>
       <c r="D11" s="1" t="n">
         <v>1</v>
@@ -5436,7 +5574,7 @@
         <v>12</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>500</v>
+        <v>511</v>
       </c>
       <c r="D12" s="1" t="n">
         <v>1</v>
@@ -5447,7 +5585,7 @@
         <v>13</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>501</v>
+        <v>512</v>
       </c>
       <c r="D13" s="1" t="n">
         <v>1</v>
@@ -5458,7 +5596,7 @@
         <v>14</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>502</v>
+        <v>513</v>
       </c>
       <c r="D14" s="1" t="n">
         <v>1</v>
@@ -5469,7 +5607,7 @@
         <v>15</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>502</v>
+        <v>513</v>
       </c>
       <c r="D15" s="1" t="n">
         <v>1</v>
@@ -5480,7 +5618,7 @@
         <v>16</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>503</v>
+        <v>514</v>
       </c>
       <c r="D16" s="1" t="n">
         <v>1</v>
@@ -5491,7 +5629,7 @@
         <v>17</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>504</v>
+        <v>515</v>
       </c>
       <c r="D17" s="1" t="n">
         <v>1</v>
@@ -5502,7 +5640,7 @@
         <v>18</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>505</v>
+        <v>516</v>
       </c>
       <c r="D18" s="1" t="n">
         <v>1</v>
@@ -5513,7 +5651,7 @@
         <v>19</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>506</v>
+        <v>517</v>
       </c>
       <c r="D19" s="1" t="n">
         <v>1</v>
@@ -5524,7 +5662,7 @@
         <v>20</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>507</v>
+        <v>518</v>
       </c>
       <c r="D20" s="1" t="n">
         <v>1</v>
@@ -5535,7 +5673,7 @@
         <v>21</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>508</v>
+        <v>519</v>
       </c>
       <c r="D21" s="1" t="n">
         <v>1</v>
@@ -5546,7 +5684,7 @@
         <v>22</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>509</v>
+        <v>520</v>
       </c>
       <c r="D22" s="1" t="n">
         <v>1</v>
@@ -5557,7 +5695,7 @@
         <v>23</v>
       </c>
       <c r="B23" s="1" t="s">
-        <v>510</v>
+        <v>521</v>
       </c>
       <c r="D23" s="1" t="n">
         <v>1</v>
@@ -5568,7 +5706,7 @@
         <v>24</v>
       </c>
       <c r="B24" s="1" t="s">
-        <v>511</v>
+        <v>522</v>
       </c>
       <c r="D24" s="1" t="n">
         <v>1</v>

</xml_diff>